<commit_message>
PKPy2 0.2.0: event-record interface for NONMEM-format data and PK/PD models
- pkpy2.Model and read_nonmem: EVID 0-4, AMT, CMT, RATE (modeled rate and
  duration), II, SS 1/2, ADDL, DVID and censoring (M3/M4)
- Structural library: one- to three-compartment disposition, zero-order and
  transit absorption, bioavailability and lag, effect compartments,
  parent-metabolite, Michaelis-Menten, TMDD, indirect response I-IV, and
  user-defined linear systems and ODEs
- Block omega, interoccasion variability, time-varying and categorical
  covariates, log-normal residuals and several outputs
- Diagnostics (EBE, PRED/IPRED, WRES/CWRES/IWRES, NPDE, shrinkage,
  simulation, VPC), sandwich covariance, profile likelihood, bootstrap, SIR,
  stepwise covariate selection and evaluate
- Examples, event-record checks in continuous integration, and the
  validation of the event-record interface in paper/event_records

The compact ModelSpec interface is unchanged.
</commit_message>
<xml_diff>
--- a/paper/raw_data/PKPy2_codebook.xlsx
+++ b/paper/raw_data/PKPy2_codebook.xlsx
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -787,6 +787,142 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>1 = passed; 0 = failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1 = first output (concentration); 2 = second output (response or metabolite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>converged</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1 = converged; 0 = not converged</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EVID</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0 = observation record; 1 = dose record</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CMT</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1 = central compartment; in oral_blq_m3, 1 = depot (doses) and 2 = central (observations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1 = dose given at steady state; 0 = other records</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CENS</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1 = below the quantification limit; 0 = quantified observation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>warfarin_pkpd: 1 = male, 0 = female; infusion_block_covariates: simulated binary covariate with reference category 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DVID</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1 = warfarin concentration (mg/L); 2 = prothrombin complex activity (%)</t>
         </is>
       </c>
     </row>
@@ -801,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3604,6 +3740,2198 @@
       </c>
       <c r="F99" t="inlineStr"/>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Prediction scenario</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>See Online Resource 1, Table S18</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>model_type</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>System type</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>linear; ODE</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Model output</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>1 = first output (concentration); 2 = second output (response or metabolite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>pkpy2</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>PKPy2 prediction</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>output units</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>rxode2</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>rxode2 prediction</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>output units</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>S10_event_prediction_checks</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>scaled_difference</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>|PKPy2 - rxode2| divided by max(|rxode2|, 1e-6 × largest value of the subject)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>quadrature = independent Gauss-Hermite quadrature at fixed parameters; compact_interface = refit through the event-record interface vs compact-interface fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Model or dataset</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>subjects</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Subjects</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>observations</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Observations</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>censored</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Censored observations</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>PKPy2 convergence status</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>converged; partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>pkpy2_ofv_bank1</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>PKPy2 OFV (bank 1 or refit)</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>-2 log L</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>pkpy2_ofv_bank2</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>PKPy2 OFV (bank 2)</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>-2 log L</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>reference_ofv</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Reference OFV (quadrature or compact interface)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>-2 log L</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>ofv_difference</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>PKPy2 minus reference</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>-2 log L</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>S11_event_likelihood_checks</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>max_relative_estimate_difference_pct</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Maximum relative difference of the estimates</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>S12_diagnostic_checks</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Diagnostic</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>PRED; IPRED; IWRES; CWRES (standardized by its own variance); NPDE (upper Cholesky factor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>S12_diagnostic_checks</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>pkpy2</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>PKPy2 value</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>S12_diagnostic_checks</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>nlmixr2</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>nlmixr2 value</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>S13_event_comparisons</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>analysis</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>infusion_block_covariates; oral_blq_m3; lognormal_residual; michaelis_menten; warfarin_pkpd</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>S13_event_comparisons</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Parameter (group:name) or exact OFV</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>theta = typical value; coefficients = covariate coefficient; omega = variance; omega_covariance = covariance; iov = interoccasion variance; sigma = residual SD</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>S13_event_comparisons</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>true_value</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Simulation value</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>as parameter</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>S13_event_comparisons</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>pkpy2</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>PKPy2 estimate or OFV</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>as parameter</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>S13_event_comparisons</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>nlmixr2_focei</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>nlmixr2 FOCEi estimate or exact OFV at its estimates</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>as parameter</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>S13_event_comparisons</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>nlmixr2_saem</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>nlmixr2 SAEM estimate or exact OFV at its estimates</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>as parameter</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>warfarin_pkpd only</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Simulation design</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>complex_linear = two-compartment steady-state infusion model; pkpd_idr = indirect-response PK/PD model</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>replicate</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Replicate</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>PKPy2 status</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>converged; partial; error</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>converged</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Convergence</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>1 = converged; 0 = not converged</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>ofv</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>OFV</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>-2 log L</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Fit time</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Parameter (group:name)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>as in S13</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>S14_event_recovery</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>as parameter</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>design</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Simulation design</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>as in S14</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>replicate</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Replicate</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>censored</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Censored observations</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>n_npde</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>NPDE values</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>npde_mean</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Mean NPDE</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>npde_variance</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>NPDE variance</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>npde_ks_p</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Kolmogorov-Smirnov p value of NPDE vs N(0, 1)</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>cwres_mean</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Mean CWRES</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>cwres_variance</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CWRES variance</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>vpc_within_CP</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Fraction of observed VPC percentiles within the 95% intervals, concentration</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>S15_event_calibration</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>vpc_within_R</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Same for the PD response</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>pkpd_idr only</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>analysis</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>theophylline_intervals; stepwise_covariates</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Reporting quantity</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>theta:CL, theta:V, theta:Ka, omega:&lt;P&gt; (variance), sigma:CP:proportional</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Interval method</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>wald; sandwich; profile; bootstrap; sir</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>estimate</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>as parameter</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>95% lower limit</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>as parameter</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>upper</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>95% upper limit</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>as parameter</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>replicate</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>SCM replicate</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Selected covariate effects</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>semicolon-separated labels parameter~covariate[form]</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>S16_interval_and_scm</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>seconds</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>SCM run time</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>CP = warfarin concentration (mg/L); R = prothrombin complex activity (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Row type</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>percentile; observation</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>bin</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Time bin</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>bin_time</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Median time of the bin, or observation time</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>quantile</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Percentile</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>0.05; 0.5; 0.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>observed</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Observed percentile or observation</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>output units</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>simulated_lower</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>2.5th percentile of the simulated percentile</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>output units</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>simulated_median</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Median of the simulated percentile</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>output units</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>S17_warfarin_pkpd_vpc</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>simulated_upper</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>97.5th percentile of the simulated percentile</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>output units</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>categorical (text)</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>as in S13</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>EVID</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Event identifier (NONMEM convention)</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>0 = observation record; 1 = dose record</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>AMT</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Dose amount</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>mg</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>0 on observation records</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>CMT</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Compartment receiving the dose or observed</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>1 = central compartment; in oral_blq_m3, 1 = depot (doses) and 2 = central (observations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>RATE</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Infusion rate</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>mg/h</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>0 = bolus or first-order input</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Dosing interval of a steady-state dose</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>0 = no steady-state dose</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>SS</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Steady-state flag</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>1 = dose given at steady state; 0 = other records</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>mg/L; % for DVID 2</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>empty on dose records; the quantification limit when CENS = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>CENS</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Censoring flag</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>1 = below the quantification limit; 0 = quantified observation</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>WT</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Body weight</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Sex</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>warfarin_pkpd: 1 = male, 0 = female; infusion_block_covariates: simulated binary covariate with reference category 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>DVID</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Observed output</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>1 = warfarin concentration (mg/L); 2 = prothrombin complex activity (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>S18_event_datasets</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add diagnostic plot examples and update manuscript materials
- examples/theophylline_diagnostics.py: NONMEM-format theophylline data through
  the event-record interface with goodness-of-fit, individual-fit and VPC plots
- examples/pkpy2_explicit_model.py: the compact-interface example of the
  manuscript supplement (Listing 1)
- pkpy2.plots: legend and axis labels for individual fits, a figure size
  option, and a VPC legend with observations drawn behind the percentiles
- README: revised article title and example list
- paper/: updated manuscript scripts, raw data (sheet S19) and example outputs
</commit_message>
<xml_diff>
--- a/paper/raw_data/PKPy2_codebook.xlsx
+++ b/paper/raw_data/PKPy2_codebook.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PKPy2: A Python framework for joint population pharmacokinetic estimation and uncertainty assessment</t>
+          <t>PKPy2: A Python framework for joint population pharmacokinetic and pharmacodynamic estimation, diagnostics, and uncertainty assessment</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -923,6 +923,23 @@
       <c r="C22" t="inlineStr">
         <is>
           <t>1 = warfarin concentration (mg/L); 2 = prothrombin complex activity (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CENS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1 = below the quantification limit; 0 = quantified observation</t>
         </is>
       </c>
     </row>
@@ -937,7 +954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F179"/>
+  <dimension ref="A1:F188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5932,6 +5949,254 @@
       </c>
       <c r="F179" t="inlineStr"/>
     </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Time after dose</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>DV</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Observed theophylline concentration</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>mg/L</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>CENS</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Censoring flag</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>categorical (numeric code)</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>1 = below the quantification limit; 0 = quantified observation</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>PRED</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Population prediction (random effects zero)</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>mg/L</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>IPRED</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Individual prediction at the conditional modes</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>mg/L</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>IWRES</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Individual weighted residual</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>CWRES</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Conditional weighted residual</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>S19_example_diagnostics</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>NPDE</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Normalized prediction distribution error</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>unitless</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>